<commit_message>
feat: fix UX for bot
</commit_message>
<xml_diff>
--- a/store/backtest_report.xlsx
+++ b/store/backtest_report.xlsx
@@ -489,7 +489,7 @@
         <v/>
       </c>
       <c r="E3" t="n">
-        <v>49.505</v>
+        <v>48.5149</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
@@ -504,7 +504,7 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>0.7311</v>
+        <v>0.6359</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
@@ -525,7 +525,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>2.1517</v>
+        <v>1.9639</v>
       </c>
       <c r="F5" t="n">
         <v>22.5543</v>
@@ -550,7 +550,7 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>-5.1423</v>
+        <v>-5.22</v>
       </c>
       <c r="F6" t="n">
         <v>-17.8404</v>
@@ -573,7 +573,7 @@
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>1.186539</v>
+        <v>1.110655</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -594,7 +594,7 @@
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>0.5207310000000001</v>
+        <v>0.479044</v>
       </c>
       <c r="F8" t="n">
         <v>1.81868</v>
@@ -619,7 +619,7 @@
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>4.4214</v>
+        <v>4.0317</v>
       </c>
       <c r="F9" t="n">
         <v>51.1841</v>
@@ -644,7 +644,7 @@
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>0.599473</v>
+        <v>0.554985</v>
       </c>
       <c r="F10" t="n">
         <v>1.903048</v>
@@ -669,7 +669,7 @@
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>0.859815</v>
+        <v>0.772352</v>
       </c>
       <c r="F11" t="n">
         <v>2.868998</v>
@@ -688,7 +688,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>32.1245</v>
+        <v>31.9566</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>[{"layer": "B0_buyhold", "sharpe": 1.8321692424745784, "cagr": 0.5536251775534435, "max_drawdown": -0.19842368333185867, "n_trades": 0}, {"layer": "fundamental", "sharpe": 1.6093930295482695, "cagr": 0.49110361326245866, "max_drawdown": -0.214859956680571, "n_trades": 0}, {"layer": "regime", "sharpe": null, "cagr": 0.0, "max_drawdown": 0.0, "n_trades": 0}, {"layer": "alpha", "sharpe": 0.8521106914728611, "cagr": 0.08236888909752338, "max_drawdown": -0.04927282879075445, "n_trades": 96}, {"layer": "risk", "sharpe": 0.5207306915927736, "cagr": 0.044213977053179754, "max_drawdown": -0.051422689765345364, "n_trades": 101}, {"layer": "B1_ta", "sharpe": 2.74139086012495, "cagr": 0.2941371053925228, "max_drawdown": -0.04288848853482574, "n_trades": 544}, {"layer": "B2_canslim", "sharpe": null, "cagr": 0.0, "max_drawdown": 0.0, "n_trades": 0}]</t>
+          <t>[{"layer": "B0_buyhold", "sharpe": 1.8321692424745784, "cagr": 0.5536251775534435, "max_drawdown": -0.19842368333185867, "n_trades": 0}, {"layer": "fundamental", "sharpe": 1.6093930295482695, "cagr": 0.49110361326245866, "max_drawdown": -0.214859956680571, "n_trades": 0}, {"layer": "regime", "sharpe": null, "cagr": 0.0, "max_drawdown": 0.0, "n_trades": 0}, {"layer": "alpha", "sharpe": 0.8521106914728611, "cagr": 0.08236888909752338, "max_drawdown": -0.04927282879075445, "n_trades": 96}, {"layer": "risk", "sharpe": 0.516597336359449, "cagr": 0.04406431880488171, "max_drawdown": -0.05140911597644471, "n_trades": 100}, {"layer": "B1_ta", "sharpe": 2.74139086012495, "cagr": 0.2941371053925228, "max_drawdown": -0.04288848853482574, "n_trades": 544}, {"layer": "B2_canslim", "sharpe": null, "cagr": 0.0, "max_drawdown": 0.0, "n_trades": 0}]</t>
         </is>
       </c>
     </row>

</xml_diff>